<commit_message>
Finalize: repo URL in CITATION, DRC event dated 2025, register note
</commit_message>
<xml_diff>
--- a/data/Supplementary_Data.xlsx
+++ b/data/Supplementary_Data.xlsx
@@ -987,82 +987,82 @@
     <t xml:space="preserve">DRC</t>
   </si>
   <si>
+    <t xml:space="preserve">2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cobalt export suspension</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Décision Nº 001/ARECOMS/2025 (22 Feb 2025), Democratic Republic of the Congo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ghana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Green Minerals Policy raw-lithium ban</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Green Minerals Policy (Ghana Cabinet, 8 Aug 2023) — policy, not a statutory instrument</t>
+  </si>
+  <si>
+    <t xml:space="preserve">local-processing mandate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guinea</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mining-licence revocations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Presidential decree revoking mining permits (Transitional Presidency), 14 May 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indonesia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Law 4/2009 domestic-processing requirement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Law No. 4 of 2009 on Mineral and Coal Mining (Indonesia), Arts. 102–104, 170</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nickel ore export ban (partial)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Government Regulation (PP) No. 1 of 2014 and MEMR Regulation No. 1 of 2014 (11 Jan 2014)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nickel ore export ban (full)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MEMR Regulation No. 11 of 2019 (nickel export ban advanced to 1 Jan 2020)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bauxite export ban</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Executive action under Law No. 3 of 2020 and GR No. 96 of 2021; effective 10 Jun 2023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mali</t>
+  </si>
+  <si>
+    <t xml:space="preserve">new mining code; state stakes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loi n°2023-040 du 29 août 2023, Code minier; Journal Officiel de la République du Mali</t>
+  </si>
+  <si>
     <t xml:space="preserve">2024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cobalt export suspension</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Décision Nº 001/ARECOMS/2025 (22 Feb 2025), DRC [see note: instrument dated 2025]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ghana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Green Minerals Policy raw-lithium ban</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Green Minerals Policy (Ghana Cabinet, 8 Aug 2023) — policy, not a statutory instrument</t>
-  </si>
-  <si>
-    <t xml:space="preserve">local-processing mandate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Guinea</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mining-licence revocations</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Presidential decree revoking mining permits (Transitional Presidency), 14 May 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Indonesia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Law 4/2009 domestic-processing requirement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Law No. 4 of 2009 on Mineral and Coal Mining (Indonesia), Arts. 102–104, 170</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2014</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nickel ore export ban (partial)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Government Regulation (PP) No. 1 of 2014 and MEMR Regulation No. 1 of 2014 (11 Jan 2014)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2020</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nickel ore export ban (full)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MEMR Regulation No. 11 of 2019 (nickel export ban advanced to 1 Jan 2020)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bauxite export ban</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Executive action under Law No. 3 of 2020 and GR No. 96 of 2021; effective 10 Jun 2023</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mali</t>
-  </si>
-  <si>
-    <t xml:space="preserve">new mining code; state stakes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Loi n°2023-040 du 29 août 2023, Code minier; Journal Officiel de la République du Mali</t>
   </si>
   <si>
     <t xml:space="preserve">Barrick/Resolute detentions; asset seizure</t>
@@ -2350,7 +2350,7 @@
         <v>325</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="C21" s="8" t="s">
         <v>280</v>
@@ -2359,18 +2359,18 @@
         <v>285</v>
       </c>
       <c r="E21" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="F21" s="6" t="s">
         <v>327</v>
-      </c>
-      <c r="F21" s="6" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
+        <v>328</v>
+      </c>
+      <c r="B22" s="8" t="s">
         <v>329</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>330</v>
       </c>
       <c r="C22" s="8" t="s">
         <v>305</v>
@@ -2379,18 +2379,18 @@
         <v>281</v>
       </c>
       <c r="E22" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="F22" s="6" t="s">
         <v>331</v>
-      </c>
-      <c r="F22" s="6" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C23" s="8" t="s">
         <v>284</v>
@@ -2399,18 +2399,18 @@
         <v>281</v>
       </c>
       <c r="E23" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="F23" s="6" t="s">
         <v>334</v>
-      </c>
-      <c r="F23" s="6" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C24" s="8" t="s">
         <v>284</v>
@@ -2419,15 +2419,15 @@
         <v>281</v>
       </c>
       <c r="E24" s="6" t="s">
+        <v>336</v>
+      </c>
+      <c r="F24" s="6" t="s">
         <v>337</v>
-      </c>
-      <c r="F24" s="6" t="s">
-        <v>338</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B25" s="8" t="s">
         <v>311</v>
@@ -2439,15 +2439,15 @@
         <v>281</v>
       </c>
       <c r="E25" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="F25" s="6" t="s">
         <v>339</v>
-      </c>
-      <c r="F25" s="6" t="s">
-        <v>340</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B26" s="8" t="s">
         <v>311</v>
@@ -2459,18 +2459,18 @@
         <v>285</v>
       </c>
       <c r="E26" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="F26" s="6" t="s">
         <v>342</v>
-      </c>
-      <c r="F26" s="6" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>318</v>
+        <v>343</v>
       </c>
       <c r="C27" s="8" t="s">
         <v>280</v>
@@ -2570,7 +2570,7 @@
         <v>357</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>318</v>
+        <v>343</v>
       </c>
       <c r="C32" s="8" t="s">
         <v>280</v>
@@ -2790,7 +2790,7 @@
         <v>377</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="C43" s="8" t="s">
         <v>288</v>
@@ -2810,7 +2810,7 @@
         <v>377</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="C44" s="8" t="s">
         <v>305</v>

</xml_diff>